<commit_message>
feat(release): v1.8.4 - resolve 25 clinical math, temperature integrity, IPC security, and web runtime defects
</commit_message>
<xml_diff>
--- a/example/bas_Result/PPP_PPG_PGA_Statistical_Summary.xlsx
+++ b/example/bas_Result/PPP_PPG_PGA_Statistical_Summary.xlsx
@@ -249,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -283,6 +283,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="2" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -296,6 +299,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="2" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -308,6 +314,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -817,32 +826,32 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>34.24</v>
+        <v>35.01</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>34.75</v>
+        <v>35.35</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>33.74</v>
+        <v>34.08</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>0.31</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.122</v>
+        <v>0.146</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.273</v>
+        <v>0.719</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.058</v>
+        <v>0.171</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>176.7</v>
+        <v>180.9</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
@@ -850,7 +859,7 @@
         </is>
       </c>
       <c r="M2" s="3" t="n">
-        <v>61.5</v>
+        <v>96.2</v>
       </c>
     </row>
     <row r="3">
@@ -866,40 +875,40 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>34.69</v>
+        <v>34.97</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>35</v>
+        <v>35.31</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>33.42</v>
+        <v>34.53</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>0.43</v>
+        <v>0.21</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>0.162</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.116</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>0.186</v>
+        <v>0.021</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>191.3</v>
+        <v>20.4</v>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>W (Medial)</t>
+          <t>E (Lateral)</t>
         </is>
       </c>
       <c r="M3" s="5" t="n">
-        <v>59.8</v>
+        <v>93.3</v>
       </c>
     </row>
     <row r="4">
@@ -915,40 +924,40 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>34.68</v>
+        <v>34.8</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>35</v>
+        <v>35.22</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>34</v>
+        <v>34.14</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.35</v>
+        <v>0.27</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.099</v>
+        <v>0.141</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.22</v>
+        <v>0.377</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.082</v>
+        <v>0.091</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>337.2</v>
+        <v>193.4</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>SE (Posterolateral)</t>
+          <t>W (Medial)</t>
         </is>
       </c>
       <c r="M4" s="3" t="n">
-        <v>93.8</v>
+        <v>65.40000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -964,40 +973,40 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>33.35</v>
+        <v>34.34</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>33.97</v>
+        <v>34.64</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>32.89</v>
+        <v>34.03</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.34</v>
+        <v>0.16</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>0.105</v>
+        <v>0.075</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>0.208</v>
+        <v>0.155</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>0.058</v>
+        <v>0.028</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>66.7</v>
+        <v>208.6</v>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>NE (Anterolateral)</t>
+          <t>SW (Posteromedial)</t>
         </is>
       </c>
       <c r="M5" s="5" t="n">
-        <v>86.59999999999999</v>
+        <v>85.90000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -1013,40 +1022,40 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>33.9</v>
+        <v>34.66</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>34</v>
+        <v>34.84</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>33.37</v>
+        <v>34.35</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.064</v>
+        <v>0.065</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.298</v>
+        <v>0.104</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.029</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>136.1</v>
+        <v>348.2</v>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>NW (Anteromedial)</t>
+          <t>E (Lateral)</t>
         </is>
       </c>
       <c r="M6" s="3" t="n">
-        <v>27.5</v>
+        <v>68.09999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -1062,40 +1071,40 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>34</v>
+        <v>34.24</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>34</v>
+        <v>34.57</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>33.88</v>
+        <v>33.69</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.01</v>
+        <v>0.22</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>0.005</v>
+        <v>0.15</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0.12</v>
+        <v>0.312</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.017</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>13.7</v>
+        <v>187.4</v>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>E (Lateral)</t>
+          <t>W (Medial)</t>
         </is>
       </c>
       <c r="M7" s="5" t="n">
-        <v>89.3</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="8">
@@ -1111,40 +1120,40 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>33.03</v>
+        <v>33.85</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>33.73</v>
+        <v>34.2</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>32.54</v>
+        <v>33.5</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.25</v>
+        <v>0.19</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.125</v>
+        <v>0.091</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0.308</v>
+        <v>0.184</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.073</v>
+        <v>0.034</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>272.2</v>
+        <v>225.1</v>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>S (Proximal / Heel)</t>
+          <t>SW (Posteromedial)</t>
         </is>
       </c>
       <c r="M8" s="3" t="n">
-        <v>33.1</v>
+        <v>47.1</v>
       </c>
     </row>
     <row r="9">
@@ -1160,40 +1169,40 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>33.31</v>
+        <v>33.76</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>33.73</v>
+        <v>34.15</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>33.01</v>
+        <v>33.57</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.21</v>
+        <v>0.16</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0.103</v>
+        <v>0.06</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>0.198</v>
+        <v>0.135</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0.048</v>
+        <v>0.04</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>57.9</v>
+        <v>356.9</v>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>NE (Anterolateral)</t>
+          <t>E (Lateral)</t>
         </is>
       </c>
       <c r="M9" s="5" t="n">
-        <v>8.300000000000001</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10">
@@ -1209,40 +1218,40 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>33.57</v>
+        <v>33.76</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>33.95</v>
+        <v>34.69</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>33.04</v>
+        <v>33.06</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.26</v>
+        <v>0.5</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.148</v>
+        <v>0.189</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.219</v>
+        <v>0.4</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.055</v>
+        <v>0.101</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>97.2</v>
+        <v>290.8</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>N (Distal / Toes)</t>
+          <t>S (Proximal / Heel)</t>
         </is>
       </c>
       <c r="M10" s="3" t="n">
-        <v>12.2</v>
+        <v>65.7</v>
       </c>
     </row>
     <row r="11">
@@ -1262,36 +1271,36 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>33.6</v>
+        <v>34.53</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>34.69</v>
+        <v>35.25</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>33</v>
+        <v>33.51</v>
       </c>
       <c r="G11" s="5" t="n">
         <v>0.5</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>0.167</v>
+        <v>0.192</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.336</v>
+        <v>0.357</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.089</v>
+        <v>0.078</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>59.9</v>
+        <v>310.2</v>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>NE (Anterolateral)</t>
+          <t>SE (Posterolateral)</t>
         </is>
       </c>
       <c r="M11" s="5" t="n">
-        <v>77.3</v>
+        <v>80.40000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -1311,36 +1320,36 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>33.99</v>
+        <v>34.25</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>34.11</v>
+        <v>34.53</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>33.92</v>
+        <v>34.09</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.02</v>
+        <v>0.11</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.013</v>
+        <v>0.078</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.095</v>
+        <v>0.157</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.016</v>
+        <v>0.032</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>144.8</v>
+        <v>190.8</v>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>NW (Anteromedial)</t>
+          <t>W (Medial)</t>
         </is>
       </c>
       <c r="M12" s="3" t="n">
-        <v>18.6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -1360,36 +1369,36 @@
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>33.9</v>
+        <v>34.32</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>34.04</v>
+        <v>34.67</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>33.4</v>
+        <v>33.78</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.17</v>
+        <v>0.28</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>0.065</v>
+        <v>0.113</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.222</v>
+        <v>0.221</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.081</v>
+        <v>0.05</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>33.8</v>
+        <v>14.2</v>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>NE (Anterolateral)</t>
+          <t>E (Lateral)</t>
         </is>
       </c>
       <c r="M13" s="5" t="n">
-        <v>33.6</v>
+        <v>66.90000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -1409,36 +1418,36 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>35.08</v>
+        <v>35.73</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>35.99</v>
+        <v>36.24</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34.03</v>
+        <v>34.07</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0.54</v>
+        <v>0.5</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.218</v>
+        <v>0.262</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0.638</v>
+        <v>1.012</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.108</v>
+        <v>0.228</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>70.7</v>
+        <v>357.6</v>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>N (Distal / Toes)</t>
+          <t>E (Lateral)</t>
         </is>
       </c>
       <c r="M14" s="3" t="n">
-        <v>60.1</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="15">
@@ -1458,36 +1467,36 @@
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>34.99</v>
+        <v>35.5</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>35.27</v>
+        <v>35.88</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>34.26</v>
+        <v>35.14</v>
       </c>
       <c r="G15" s="5" t="n">
         <v>0.13</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>0.057</v>
+        <v>0.094</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>0.503</v>
+        <v>0.461</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>0.093</v>
+        <v>0.074</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>145.4</v>
+        <v>223.7</v>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>NW (Anteromedial)</t>
+          <t>SW (Posteromedial)</t>
         </is>
       </c>
       <c r="M15" s="5" t="n">
-        <v>21.5</v>
+        <v>33.1</v>
       </c>
     </row>
     <row r="16">
@@ -1507,28 +1516,28 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>34.97</v>
+        <v>35.52</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>35.11</v>
+        <v>35.85</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>34.42</v>
+        <v>34.98</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0.14</v>
+        <v>0.26</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.065</v>
+        <v>0.102</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>0.216</v>
+        <v>0.168</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.058</v>
+        <v>0.041</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>15.1</v>
+        <v>2</v>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
@@ -1536,7 +1545,7 @@
         </is>
       </c>
       <c r="M16" s="3" t="n">
-        <v>27.8</v>
+        <v>70.3</v>
       </c>
     </row>
     <row r="17">
@@ -1556,36 +1565,36 @@
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>35.7</v>
+        <v>36.42</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>36.2</v>
+        <v>36.89</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>34.46</v>
+        <v>35.47</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0.38</v>
+        <v>0.34</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>0.208</v>
+        <v>0.253</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.629</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.144</v>
+        <v>0.159</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>106.2</v>
+        <v>318.6</v>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>N (Distal / Toes)</t>
+          <t>SE (Posterolateral)</t>
         </is>
       </c>
       <c r="M17" s="5" t="n">
-        <v>34.4</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="18">
@@ -1605,36 +1614,36 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>35.15</v>
+        <v>35.64</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>35.92</v>
+        <v>36.21</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>34.49</v>
+        <v>34.74</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>0.35</v>
+        <v>0.38</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0.152</v>
+        <v>0.191</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>0.316</v>
+        <v>0.548</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.166</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>216.9</v>
+        <v>165.4</v>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>SW (Posteromedial)</t>
+          <t>W (Medial)</t>
         </is>
       </c>
       <c r="M18" s="3" t="n">
-        <v>73.40000000000001</v>
+        <v>87.5</v>
       </c>
     </row>
     <row r="19">
@@ -1654,36 +1663,36 @@
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>35.65</v>
+        <v>36.04</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>35.99</v>
+        <v>36.35</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>35.13</v>
+        <v>35.53</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>0.152</v>
+        <v>0.116</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>0.217</v>
+        <v>0.192</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.057</v>
+        <v>0.042</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>277.9</v>
+        <v>27.3</v>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>S (Proximal / Heel)</t>
+          <t>NE (Anterolateral)</t>
         </is>
       </c>
       <c r="M19" s="5" t="n">
-        <v>27.5</v>
+        <v>49.4</v>
       </c>
     </row>
     <row r="20">
@@ -1703,36 +1712,36 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>34.78</v>
+        <v>36</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>35.98</v>
+        <v>36.78</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>33.33</v>
+        <v>34.5</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>0.7</v>
+        <v>0.64</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0.262</v>
+        <v>0.315</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>0.711</v>
+        <v>0.881</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.104</v>
+        <v>0.191</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>60.2</v>
+        <v>335.5</v>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>NE (Anterolateral)</t>
+          <t>SE (Posterolateral)</t>
         </is>
       </c>
       <c r="M20" s="3" t="n">
-        <v>77.2</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21">
@@ -1752,36 +1761,36 @@
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>35.09</v>
+        <v>35.69</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>35.71</v>
+        <v>36.16</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>34.58</v>
+        <v>34.94</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="H21" s="5" t="n">
+        <v>0.148</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>0.551</v>
+      </c>
+      <c r="J21" s="5" t="n">
         <v>0.116</v>
       </c>
-      <c r="I21" s="5" t="n">
-        <v>0.339</v>
-      </c>
-      <c r="J21" s="5" t="n">
-        <v>0.083</v>
-      </c>
       <c r="K21" s="5" t="n">
-        <v>78</v>
+        <v>227.5</v>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>N (Distal / Toes)</t>
+          <t>SW (Posteromedial)</t>
         </is>
       </c>
       <c r="M21" s="5" t="n">
-        <v>31.4</v>
+        <v>41.8</v>
       </c>
     </row>
     <row r="22">
@@ -1801,36 +1810,36 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>35.31</v>
+        <v>35.83</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>35.83</v>
+        <v>36.24</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>34.77</v>
+        <v>35.11</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>0.28</v>
+        <v>0.25</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.129</v>
+        <v>0.136</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>0.233</v>
+        <v>0.252</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.061</v>
+        <v>0.044</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>117.3</v>
+        <v>275.9</v>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>NW (Anteromedial)</t>
+          <t>S (Proximal / Heel)</t>
         </is>
       </c>
       <c r="M22" s="3" t="n">
-        <v>40.5</v>
+        <v>44.9</v>
       </c>
     </row>
     <row r="25" ht="26" customHeight="1">
@@ -1895,26 +1904,27 @@
           <t>Kolom D (D2:D22)</t>
         </is>
       </c>
-      <c r="D27" s="11">
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>'=AVERAGE(D2:D22)</t>
+        </is>
+      </c>
+      <c r="E27" s="14">
         <f>AVERAGE(D2:D22)</f>
         <v/>
       </c>
-      <c r="E27" s="13">
-        <f>AVERAGE(D2:D22)</f>
-        <v/>
-      </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
           <t>T1 (Hallux), M1 &amp; M2 (Metatarsal) adalah titik kontak beban tumpuan puncak fase berjalan (stance phase). Rata-rata suhu mencerminkan perfusi basal jaringan kulit.</t>
         </is>
       </c>
-      <c r="G27" s="14" t="n"/>
-      <c r="H27" s="14" t="n"/>
-      <c r="I27" s="14" t="n"/>
-      <c r="J27" s="14" t="n"/>
-      <c r="K27" s="14" t="n"/>
-      <c r="L27" s="14" t="n"/>
-      <c r="M27" s="14" t="n"/>
+      <c r="G27" s="15" t="n"/>
+      <c r="H27" s="15" t="n"/>
+      <c r="I27" s="15" t="n"/>
+      <c r="J27" s="15" t="n"/>
+      <c r="K27" s="15" t="n"/>
+      <c r="L27" s="15" t="n"/>
+      <c r="M27" s="15" t="n"/>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="10" t="inlineStr">
@@ -1932,26 +1942,27 @@
           <t>Kolom E (E2:E22)</t>
         </is>
       </c>
-      <c r="D28" s="11">
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>'=MAX(E2:E22)</t>
+        </is>
+      </c>
+      <c r="E28" s="14">
         <f>MAX(E2:E22)</f>
         <v/>
       </c>
-      <c r="E28" s="13">
-        <f>MAX(E2:E22)</f>
-        <v/>
-      </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
           <t>Hotspot lokal adalah penanda awal hiperemia dan mikrotrauma jaringan dalam sebelum timbul kerusakan kulit terbuka (ulkus diabetik).</t>
         </is>
       </c>
-      <c r="G28" s="14" t="n"/>
-      <c r="H28" s="14" t="n"/>
-      <c r="I28" s="14" t="n"/>
-      <c r="J28" s="14" t="n"/>
-      <c r="K28" s="14" t="n"/>
-      <c r="L28" s="14" t="n"/>
-      <c r="M28" s="14" t="n"/>
+      <c r="G28" s="15" t="n"/>
+      <c r="H28" s="15" t="n"/>
+      <c r="I28" s="15" t="n"/>
+      <c r="J28" s="15" t="n"/>
+      <c r="K28" s="15" t="n"/>
+      <c r="L28" s="15" t="n"/>
+      <c r="M28" s="15" t="n"/>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
@@ -1969,213 +1980,217 @@
           <t>Kolom F (F2:F22)</t>
         </is>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>'=MIN(F2:F22)</t>
+        </is>
+      </c>
+      <c r="E29" s="14">
         <f>MIN(F2:F22)</f>
         <v/>
       </c>
-      <c r="E29" s="13">
-        <f>MIN(F2:F22)</f>
-        <v/>
-      </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
           <t>Mengevaluasi batas bawah suhu untuk skrining hipoperfusi atau iskemia akibat Peripheral Artery Disease (PAD).</t>
         </is>
       </c>
-      <c r="G29" s="14" t="n"/>
-      <c r="H29" s="14" t="n"/>
-      <c r="I29" s="14" t="n"/>
-      <c r="J29" s="14" t="n"/>
-      <c r="K29" s="14" t="n"/>
-      <c r="L29" s="14" t="n"/>
-      <c r="M29" s="14" t="n"/>
+      <c r="G29" s="15" t="n"/>
+      <c r="H29" s="15" t="n"/>
+      <c r="I29" s="15" t="n"/>
+      <c r="J29" s="15" t="n"/>
+      <c r="K29" s="15" t="n"/>
+      <c r="L29" s="15" t="n"/>
+      <c r="M29" s="15" t="n"/>
     </row>
     <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>PPG (Mean Gradient)</t>
         </is>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>Seberapa tajam rata-rata lonjakan perbedaan suhu spasial?</t>
         </is>
       </c>
-      <c r="C30" s="17" t="inlineStr">
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>Kolom H (H2:H22)</t>
         </is>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>'=AVERAGE(H2:H22)</t>
+        </is>
+      </c>
+      <c r="E30" s="20">
         <f>AVERAGE(H2:H22)</f>
         <v/>
       </c>
-      <c r="E30" s="18">
-        <f>AVERAGE(H2:H22)</f>
-        <v/>
-      </c>
-      <c r="F30" s="16" t="inlineStr">
+      <c r="F30" s="17" t="inlineStr">
         <is>
           <t>Membedakan hangat fisiologis merata (suhu ruang/aktivitas) vs peradangan fokal aktif. Gradien tinggi menandakan batas radang aktif.</t>
         </is>
       </c>
-      <c r="G30" s="19" t="n"/>
-      <c r="H30" s="19" t="n"/>
-      <c r="I30" s="19" t="n"/>
-      <c r="J30" s="19" t="n"/>
-      <c r="K30" s="19" t="n"/>
-      <c r="L30" s="19" t="n"/>
-      <c r="M30" s="19" t="n"/>
+      <c r="G30" s="21" t="n"/>
+      <c r="H30" s="21" t="n"/>
+      <c r="I30" s="21" t="n"/>
+      <c r="J30" s="21" t="n"/>
+      <c r="K30" s="21" t="n"/>
+      <c r="L30" s="21" t="n"/>
+      <c r="M30" s="21" t="n"/>
     </row>
     <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>PPG (Peak Gradient)</t>
         </is>
       </c>
-      <c r="B31" s="16" t="inlineStr">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>Seberapa curam batas kontras panas paling tajam di titik radang?</t>
         </is>
       </c>
-      <c r="C31" s="17" t="inlineStr">
+      <c r="C31" s="18" t="inlineStr">
         <is>
           <t>Kolom I (I2:I22)</t>
         </is>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>'=MAX(I2:I22)</t>
+        </is>
+      </c>
+      <c r="E31" s="20">
         <f>MAX(I2:I22)</f>
         <v/>
       </c>
-      <c r="E31" s="18">
-        <f>MAX(I2:I22)</f>
-        <v/>
-      </c>
-      <c r="F31" s="16" t="inlineStr">
+      <c r="F31" s="17" t="inlineStr">
         <is>
           <t>Puncak gradien melokalisir batas tepi fokal infeksi dalam atau deformitas Charcot Foot sebelum luka terlihat kasat mata.</t>
         </is>
       </c>
-      <c r="G31" s="19" t="n"/>
-      <c r="H31" s="19" t="n"/>
-      <c r="I31" s="19" t="n"/>
-      <c r="J31" s="19" t="n"/>
-      <c r="K31" s="19" t="n"/>
-      <c r="L31" s="19" t="n"/>
-      <c r="M31" s="19" t="n"/>
+      <c r="G31" s="21" t="n"/>
+      <c r="H31" s="21" t="n"/>
+      <c r="I31" s="21" t="n"/>
+      <c r="J31" s="21" t="n"/>
+      <c r="K31" s="21" t="n"/>
+      <c r="L31" s="21" t="n"/>
+      <c r="M31" s="21" t="n"/>
     </row>
     <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="20" t="inlineStr">
+      <c r="A32" s="22" t="inlineStr">
         <is>
           <t>PGA (Mean Angle)</t>
         </is>
       </c>
-      <c r="B32" s="21" t="inlineStr">
+      <c r="B32" s="23" t="inlineStr">
         <is>
           <t>Ke sudut berapa derajat vektor rambatan panas mengalir?</t>
         </is>
       </c>
-      <c r="C32" s="22" t="inlineStr">
+      <c r="C32" s="24" t="inlineStr">
         <is>
           <t>Kolom K (K2:K22)</t>
         </is>
       </c>
-      <c r="D32" s="21">
-        <f>AVERAGE(K2:K22)</f>
-        <v/>
-      </c>
-      <c r="E32" s="23">
-        <f>AVERAGE(K2:K22)</f>
-        <v/>
-      </c>
-      <c r="F32" s="21" t="inlineStr">
+      <c r="D32" s="25" t="inlineStr">
+        <is>
+          <t>Rata-rata Sirkular Vektor (Weighted Circular Mean)</t>
+        </is>
+      </c>
+      <c r="E32" s="26" t="n">
+        <v>295.25</v>
+      </c>
+      <c r="F32" s="23" t="inlineStr">
         <is>
           <t>Menentukan orientasi jalur penyebaran kalor dari titik tumpuan metatarsal ke jaringan sekitar.</t>
         </is>
       </c>
-      <c r="G32" s="24" t="n"/>
-      <c r="H32" s="24" t="n"/>
-      <c r="I32" s="24" t="n"/>
-      <c r="J32" s="24" t="n"/>
-      <c r="K32" s="24" t="n"/>
-      <c r="L32" s="24" t="n"/>
-      <c r="M32" s="24" t="n"/>
+      <c r="G32" s="27" t="n"/>
+      <c r="H32" s="27" t="n"/>
+      <c r="I32" s="27" t="n"/>
+      <c r="J32" s="27" t="n"/>
+      <c r="K32" s="27" t="n"/>
+      <c r="L32" s="27" t="n"/>
+      <c r="M32" s="27" t="n"/>
     </row>
     <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="20" t="inlineStr">
+      <c r="A33" s="22" t="inlineStr">
         <is>
           <t>PGA (Direction Compass)</t>
         </is>
       </c>
-      <c r="B33" s="21" t="inlineStr">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>Ke arah anatomis mana panas merambat pada kaki pasien?</t>
         </is>
       </c>
-      <c r="C33" s="22" t="inlineStr">
+      <c r="C33" s="24" t="inlineStr">
         <is>
           <t>Kolom L (L2:L22)</t>
         </is>
       </c>
-      <c r="D33" s="21" t="inlineStr">
+      <c r="D33" s="25" t="inlineStr">
         <is>
           <t>Konversi 8 arah kardinal</t>
         </is>
       </c>
-      <c r="E33" s="25" t="inlineStr">
+      <c r="E33" s="28" t="inlineStr">
         <is>
           <t>Lihat Kolom L per baris</t>
         </is>
       </c>
-      <c r="F33" s="21" t="inlineStr">
+      <c r="F33" s="23" t="inlineStr">
         <is>
           <t>Memandu klinisi apakah panas menjalar ke sela jari kaki (interdigital), ke arkus medial, atau ke lateral luar.</t>
         </is>
       </c>
-      <c r="G33" s="24" t="n"/>
-      <c r="H33" s="24" t="n"/>
-      <c r="I33" s="24" t="n"/>
-      <c r="J33" s="24" t="n"/>
-      <c r="K33" s="24" t="n"/>
-      <c r="L33" s="24" t="n"/>
-      <c r="M33" s="24" t="n"/>
+      <c r="G33" s="27" t="n"/>
+      <c r="H33" s="27" t="n"/>
+      <c r="I33" s="27" t="n"/>
+      <c r="J33" s="27" t="n"/>
+      <c r="K33" s="27" t="n"/>
+      <c r="L33" s="27" t="n"/>
+      <c r="M33" s="27" t="n"/>
     </row>
     <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="20" t="inlineStr">
+      <c r="A34" s="22" t="inlineStr">
         <is>
           <t>PGA (Vector Coherence %)</t>
         </is>
       </c>
-      <c r="B34" s="21" t="inlineStr">
+      <c r="B34" s="23" t="inlineStr">
         <is>
           <t>Seberapa seragam arah aliran rambatan panas (0-100%)?</t>
         </is>
       </c>
-      <c r="C34" s="22" t="inlineStr">
+      <c r="C34" s="24" t="inlineStr">
         <is>
           <t>Kolom M (M2:M22)</t>
         </is>
       </c>
-      <c r="D34" s="21">
+      <c r="D34" s="25" t="inlineStr">
+        <is>
+          <t>'=AVERAGE(M2:M22)</t>
+        </is>
+      </c>
+      <c r="E34" s="26">
         <f>AVERAGE(M2:M22)</f>
         <v/>
       </c>
-      <c r="E34" s="23">
-        <f>AVERAGE(M2:M22)</f>
-        <v/>
-      </c>
-      <c r="F34" s="21" t="inlineStr">
+      <c r="F34" s="23" t="inlineStr">
         <is>
           <t>Koherensi tinggi (&gt;75%) membuktikan disipasi panas terarah kuat (fokus vaskular); koherensi rendah (&lt;50%) berarti difusi acak normal.</t>
         </is>
       </c>
-      <c r="G34" s="24" t="n"/>
-      <c r="H34" s="24" t="n"/>
-      <c r="I34" s="24" t="n"/>
-      <c r="J34" s="24" t="n"/>
-      <c r="K34" s="24" t="n"/>
-      <c r="L34" s="24" t="n"/>
-      <c r="M34" s="24" t="n"/>
+      <c r="G34" s="27" t="n"/>
+      <c r="H34" s="27" t="n"/>
+      <c r="I34" s="27" t="n"/>
+      <c r="J34" s="27" t="n"/>
+      <c r="K34" s="27" t="n"/>
+      <c r="L34" s="27" t="n"/>
+      <c r="M34" s="27" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -2229,119 +2244,119 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Image_Name</t>
         </is>
       </c>
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="29" t="inlineStr">
         <is>
           <t>Foot_Side</t>
         </is>
       </c>
-      <c r="C1" s="26" t="inlineStr">
+      <c r="C1" s="29" t="inlineStr">
+        <is>
+          <t>M1_PPP_Mean_C</t>
+        </is>
+      </c>
+      <c r="D1" s="29" t="inlineStr">
+        <is>
+          <t>M1_PPP_Peak_C</t>
+        </is>
+      </c>
+      <c r="E1" s="29" t="inlineStr">
+        <is>
+          <t>M1_PPG_Mean_Grad</t>
+        </is>
+      </c>
+      <c r="F1" s="29" t="inlineStr">
+        <is>
+          <t>M1_PPG_Peak_Grad</t>
+        </is>
+      </c>
+      <c r="G1" s="29" t="inlineStr">
+        <is>
+          <t>M1_PGA_Angle_Deg</t>
+        </is>
+      </c>
+      <c r="H1" s="29" t="inlineStr">
+        <is>
+          <t>M1_PGA_Direction</t>
+        </is>
+      </c>
+      <c r="I1" s="29" t="inlineStr">
+        <is>
+          <t>M1_PGA_Coherence_Pct</t>
+        </is>
+      </c>
+      <c r="J1" s="29" t="inlineStr">
+        <is>
+          <t>M2_PPP_Mean_C</t>
+        </is>
+      </c>
+      <c r="K1" s="29" t="inlineStr">
+        <is>
+          <t>M2_PPP_Peak_C</t>
+        </is>
+      </c>
+      <c r="L1" s="29" t="inlineStr">
+        <is>
+          <t>M2_PPG_Mean_Grad</t>
+        </is>
+      </c>
+      <c r="M1" s="29" t="inlineStr">
+        <is>
+          <t>M2_PPG_Peak_Grad</t>
+        </is>
+      </c>
+      <c r="N1" s="29" t="inlineStr">
+        <is>
+          <t>M2_PGA_Angle_Deg</t>
+        </is>
+      </c>
+      <c r="O1" s="29" t="inlineStr">
+        <is>
+          <t>M2_PGA_Direction</t>
+        </is>
+      </c>
+      <c r="P1" s="29" t="inlineStr">
+        <is>
+          <t>M2_PGA_Coherence_Pct</t>
+        </is>
+      </c>
+      <c r="Q1" s="29" t="inlineStr">
         <is>
           <t>T1_PPP_Mean_C</t>
         </is>
       </c>
-      <c r="D1" s="26" t="inlineStr">
+      <c r="R1" s="29" t="inlineStr">
         <is>
           <t>T1_PPP_Peak_C</t>
         </is>
       </c>
-      <c r="E1" s="26" t="inlineStr">
+      <c r="S1" s="29" t="inlineStr">
         <is>
           <t>T1_PPG_Mean_Grad</t>
         </is>
       </c>
-      <c r="F1" s="26" t="inlineStr">
+      <c r="T1" s="29" t="inlineStr">
         <is>
           <t>T1_PPG_Peak_Grad</t>
         </is>
       </c>
-      <c r="G1" s="26" t="inlineStr">
+      <c r="U1" s="29" t="inlineStr">
         <is>
           <t>T1_PGA_Angle_Deg</t>
         </is>
       </c>
-      <c r="H1" s="26" t="inlineStr">
+      <c r="V1" s="29" t="inlineStr">
         <is>
           <t>T1_PGA_Direction</t>
         </is>
       </c>
-      <c r="I1" s="26" t="inlineStr">
+      <c r="W1" s="29" t="inlineStr">
         <is>
           <t>T1_PGA_Coherence_Pct</t>
-        </is>
-      </c>
-      <c r="J1" s="26" t="inlineStr">
-        <is>
-          <t>M1_PPP_Mean_C</t>
-        </is>
-      </c>
-      <c r="K1" s="26" t="inlineStr">
-        <is>
-          <t>M1_PPP_Peak_C</t>
-        </is>
-      </c>
-      <c r="L1" s="26" t="inlineStr">
-        <is>
-          <t>M1_PPG_Mean_Grad</t>
-        </is>
-      </c>
-      <c r="M1" s="26" t="inlineStr">
-        <is>
-          <t>M1_PPG_Peak_Grad</t>
-        </is>
-      </c>
-      <c r="N1" s="26" t="inlineStr">
-        <is>
-          <t>M1_PGA_Angle_Deg</t>
-        </is>
-      </c>
-      <c r="O1" s="26" t="inlineStr">
-        <is>
-          <t>M1_PGA_Direction</t>
-        </is>
-      </c>
-      <c r="P1" s="26" t="inlineStr">
-        <is>
-          <t>M1_PGA_Coherence_Pct</t>
-        </is>
-      </c>
-      <c r="Q1" s="26" t="inlineStr">
-        <is>
-          <t>M2_PPP_Mean_C</t>
-        </is>
-      </c>
-      <c r="R1" s="26" t="inlineStr">
-        <is>
-          <t>M2_PPP_Peak_C</t>
-        </is>
-      </c>
-      <c r="S1" s="26" t="inlineStr">
-        <is>
-          <t>M2_PPG_Mean_Grad</t>
-        </is>
-      </c>
-      <c r="T1" s="26" t="inlineStr">
-        <is>
-          <t>M2_PPG_Peak_Grad</t>
-        </is>
-      </c>
-      <c r="U1" s="26" t="inlineStr">
-        <is>
-          <t>M2_PGA_Angle_Deg</t>
-        </is>
-      </c>
-      <c r="V1" s="26" t="inlineStr">
-        <is>
-          <t>M2_PGA_Direction</t>
-        </is>
-      </c>
-      <c r="W1" s="26" t="inlineStr">
-        <is>
-          <t>M2_PGA_Coherence_Pct</t>
         </is>
       </c>
     </row>
@@ -2357,19 +2372,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>34.24</v>
+        <v>35.01</v>
       </c>
       <c r="D2" t="n">
-        <v>34.75</v>
+        <v>35.35</v>
       </c>
       <c r="E2" t="n">
-        <v>0.122</v>
+        <v>0.146</v>
       </c>
       <c r="F2" t="n">
-        <v>0.273</v>
+        <v>0.719</v>
       </c>
       <c r="G2" t="n">
-        <v>176.7</v>
+        <v>180.9</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -2377,53 +2392,53 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>61.5</v>
+        <v>96.2</v>
       </c>
       <c r="J2" t="n">
-        <v>34.69</v>
+        <v>34.97</v>
       </c>
       <c r="K2" t="n">
-        <v>35</v>
+        <v>35.31</v>
       </c>
       <c r="L2" t="n">
-        <v>0.162</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="M2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.116</v>
       </c>
       <c r="N2" t="n">
-        <v>191.3</v>
+        <v>20.4</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>E (Lateral)</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>93.3</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="R2" t="n">
+        <v>35.22</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.141</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.377</v>
+      </c>
+      <c r="U2" t="n">
+        <v>193.4</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
           <t>W (Medial)</t>
         </is>
       </c>
-      <c r="P2" t="n">
-        <v>59.8</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>34.68</v>
-      </c>
-      <c r="R2" t="n">
-        <v>35</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.099</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="U2" t="n">
-        <v>337.2</v>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>SE (Posterolateral)</t>
-        </is>
-      </c>
       <c r="W2" t="n">
-        <v>93.8</v>
+        <v>65.40000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -2438,73 +2453,73 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>33.35</v>
+        <v>34.34</v>
       </c>
       <c r="D3" t="n">
-        <v>33.97</v>
+        <v>34.64</v>
       </c>
       <c r="E3" t="n">
-        <v>0.105</v>
+        <v>0.075</v>
       </c>
       <c r="F3" t="n">
-        <v>0.208</v>
+        <v>0.155</v>
       </c>
       <c r="G3" t="n">
-        <v>66.7</v>
+        <v>208.6</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NE (Anterolateral)</t>
+          <t>SW (Posteromedial)</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>86.59999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>33.9</v>
+        <v>34.66</v>
       </c>
       <c r="K3" t="n">
-        <v>34</v>
+        <v>34.84</v>
       </c>
       <c r="L3" t="n">
-        <v>0.064</v>
+        <v>0.065</v>
       </c>
       <c r="M3" t="n">
-        <v>0.298</v>
+        <v>0.104</v>
       </c>
       <c r="N3" t="n">
-        <v>136.1</v>
+        <v>348.2</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>NW (Anteromedial)</t>
+          <t>E (Lateral)</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>27.5</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>34</v>
+        <v>34.24</v>
       </c>
       <c r="R3" t="n">
-        <v>34</v>
+        <v>34.57</v>
       </c>
       <c r="S3" t="n">
-        <v>0.005</v>
+        <v>0.15</v>
       </c>
       <c r="T3" t="n">
-        <v>0.12</v>
+        <v>0.312</v>
       </c>
       <c r="U3" t="n">
-        <v>13.7</v>
+        <v>187.4</v>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>E (Lateral)</t>
+          <t>W (Medial)</t>
         </is>
       </c>
       <c r="W3" t="n">
-        <v>89.3</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="4">
@@ -2519,73 +2534,73 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>33.03</v>
+        <v>33.85</v>
       </c>
       <c r="D4" t="n">
-        <v>33.73</v>
+        <v>34.2</v>
       </c>
       <c r="E4" t="n">
-        <v>0.125</v>
+        <v>0.091</v>
       </c>
       <c r="F4" t="n">
-        <v>0.308</v>
+        <v>0.184</v>
       </c>
       <c r="G4" t="n">
-        <v>272.2</v>
+        <v>225.1</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>SW (Posteromedial)</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>33.76</v>
+      </c>
+      <c r="K4" t="n">
+        <v>34.15</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="N4" t="n">
+        <v>356.9</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>E (Lateral)</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>90</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>33.76</v>
+      </c>
+      <c r="R4" t="n">
+        <v>34.69</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="U4" t="n">
+        <v>290.8</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
           <t>S (Proximal / Heel)</t>
         </is>
       </c>
-      <c r="I4" t="n">
-        <v>33.1</v>
-      </c>
-      <c r="J4" t="n">
-        <v>33.31</v>
-      </c>
-      <c r="K4" t="n">
-        <v>33.73</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.103</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.198</v>
-      </c>
-      <c r="N4" t="n">
-        <v>57.9</v>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>NE (Anterolateral)</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>33.57</v>
-      </c>
-      <c r="R4" t="n">
-        <v>33.95</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0.148</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0.219</v>
-      </c>
-      <c r="U4" t="n">
-        <v>97.2</v>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>N (Distal / Toes)</t>
-        </is>
-      </c>
       <c r="W4" t="n">
-        <v>12.2</v>
+        <v>65.7</v>
       </c>
     </row>
     <row r="5">
@@ -2600,73 +2615,73 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>33.6</v>
+        <v>34.25</v>
       </c>
       <c r="D5" t="n">
-        <v>34.69</v>
+        <v>34.53</v>
       </c>
       <c r="E5" t="n">
-        <v>0.167</v>
+        <v>0.078</v>
       </c>
       <c r="F5" t="n">
-        <v>0.336</v>
+        <v>0.157</v>
       </c>
       <c r="G5" t="n">
-        <v>59.9</v>
+        <v>190.8</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NE (Anterolateral)</t>
+          <t>W (Medial)</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>77.3</v>
+        <v>8</v>
       </c>
       <c r="J5" t="n">
-        <v>33.99</v>
+        <v>34.32</v>
       </c>
       <c r="K5" t="n">
-        <v>34.11</v>
+        <v>34.67</v>
       </c>
       <c r="L5" t="n">
-        <v>0.013</v>
+        <v>0.113</v>
       </c>
       <c r="M5" t="n">
-        <v>0.095</v>
+        <v>0.221</v>
       </c>
       <c r="N5" t="n">
-        <v>144.8</v>
+        <v>14.2</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>NW (Anteromedial)</t>
+          <t>E (Lateral)</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>18.6</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="Q5" t="n">
-        <v>33.9</v>
+        <v>34.53</v>
       </c>
       <c r="R5" t="n">
-        <v>34.04</v>
+        <v>35.25</v>
       </c>
       <c r="S5" t="n">
-        <v>0.065</v>
+        <v>0.192</v>
       </c>
       <c r="T5" t="n">
-        <v>0.222</v>
+        <v>0.357</v>
       </c>
       <c r="U5" t="n">
-        <v>33.8</v>
+        <v>310.2</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>NE (Anterolateral)</t>
+          <t>SE (Posterolateral)</t>
         </is>
       </c>
       <c r="W5" t="n">
-        <v>33.6</v>
+        <v>80.40000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -2681,65 +2696,65 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>35.08</v>
+        <v>35.5</v>
       </c>
       <c r="D6" t="n">
-        <v>35.99</v>
+        <v>35.88</v>
       </c>
       <c r="E6" t="n">
-        <v>0.218</v>
+        <v>0.094</v>
       </c>
       <c r="F6" t="n">
-        <v>0.638</v>
+        <v>0.461</v>
       </c>
       <c r="G6" t="n">
-        <v>70.7</v>
+        <v>223.7</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>N (Distal / Toes)</t>
+          <t>SW (Posteromedial)</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>60.1</v>
+        <v>33.1</v>
       </c>
       <c r="J6" t="n">
-        <v>34.99</v>
+        <v>35.52</v>
       </c>
       <c r="K6" t="n">
-        <v>35.27</v>
+        <v>35.85</v>
       </c>
       <c r="L6" t="n">
-        <v>0.057</v>
+        <v>0.102</v>
       </c>
       <c r="M6" t="n">
-        <v>0.503</v>
+        <v>0.168</v>
       </c>
       <c r="N6" t="n">
-        <v>145.4</v>
+        <v>2</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>NW (Anteromedial)</t>
+          <t>E (Lateral)</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>21.5</v>
+        <v>70.3</v>
       </c>
       <c r="Q6" t="n">
-        <v>34.97</v>
+        <v>35.73</v>
       </c>
       <c r="R6" t="n">
-        <v>35.11</v>
+        <v>36.24</v>
       </c>
       <c r="S6" t="n">
-        <v>0.065</v>
+        <v>0.262</v>
       </c>
       <c r="T6" t="n">
-        <v>0.216</v>
+        <v>1.012</v>
       </c>
       <c r="U6" t="n">
-        <v>15.1</v>
+        <v>357.6</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
@@ -2747,7 +2762,7 @@
         </is>
       </c>
       <c r="W6" t="n">
-        <v>27.8</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -2762,73 +2777,73 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>35.7</v>
+        <v>35.64</v>
       </c>
       <c r="D7" t="n">
-        <v>36.2</v>
+        <v>36.21</v>
       </c>
       <c r="E7" t="n">
-        <v>0.208</v>
+        <v>0.191</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.548</v>
       </c>
       <c r="G7" t="n">
-        <v>106.2</v>
+        <v>165.4</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>N (Distal / Toes)</t>
+          <t>W (Medial)</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>34.4</v>
+        <v>87.5</v>
       </c>
       <c r="J7" t="n">
-        <v>35.15</v>
+        <v>36.04</v>
       </c>
       <c r="K7" t="n">
-        <v>35.92</v>
+        <v>36.35</v>
       </c>
       <c r="L7" t="n">
-        <v>0.152</v>
+        <v>0.116</v>
       </c>
       <c r="M7" t="n">
-        <v>0.316</v>
+        <v>0.192</v>
       </c>
       <c r="N7" t="n">
-        <v>216.9</v>
+        <v>27.3</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>SW (Posteromedial)</t>
+          <t>NE (Anterolateral)</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>73.40000000000001</v>
+        <v>49.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>35.65</v>
+        <v>36.42</v>
       </c>
       <c r="R7" t="n">
-        <v>35.99</v>
+        <v>36.89</v>
       </c>
       <c r="S7" t="n">
-        <v>0.152</v>
+        <v>0.253</v>
       </c>
       <c r="T7" t="n">
-        <v>0.217</v>
+        <v>0.629</v>
       </c>
       <c r="U7" t="n">
-        <v>277.9</v>
+        <v>318.6</v>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>S (Proximal / Heel)</t>
+          <t>SE (Posterolateral)</t>
         </is>
       </c>
       <c r="W7" t="n">
-        <v>27.5</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="8">
@@ -2843,73 +2858,73 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>34.78</v>
+        <v>35.69</v>
       </c>
       <c r="D8" t="n">
-        <v>35.98</v>
+        <v>36.16</v>
       </c>
       <c r="E8" t="n">
-        <v>0.262</v>
+        <v>0.148</v>
       </c>
       <c r="F8" t="n">
-        <v>0.711</v>
+        <v>0.551</v>
       </c>
       <c r="G8" t="n">
-        <v>60.2</v>
+        <v>227.5</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NE (Anterolateral)</t>
+          <t>SW (Posteromedial)</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>77.2</v>
+        <v>41.8</v>
       </c>
       <c r="J8" t="n">
-        <v>35.09</v>
+        <v>35.83</v>
       </c>
       <c r="K8" t="n">
-        <v>35.71</v>
+        <v>36.24</v>
       </c>
       <c r="L8" t="n">
-        <v>0.116</v>
+        <v>0.136</v>
       </c>
       <c r="M8" t="n">
-        <v>0.339</v>
+        <v>0.252</v>
       </c>
       <c r="N8" t="n">
-        <v>78</v>
+        <v>275.9</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>N (Distal / Toes)</t>
+          <t>S (Proximal / Heel)</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>31.4</v>
+        <v>44.9</v>
       </c>
       <c r="Q8" t="n">
-        <v>35.31</v>
+        <v>36</v>
       </c>
       <c r="R8" t="n">
-        <v>35.83</v>
+        <v>36.78</v>
       </c>
       <c r="S8" t="n">
-        <v>0.129</v>
+        <v>0.315</v>
       </c>
       <c r="T8" t="n">
-        <v>0.233</v>
+        <v>0.881</v>
       </c>
       <c r="U8" t="n">
-        <v>117.3</v>
+        <v>335.5</v>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>NW (Anteromedial)</t>
+          <t>SE (Posterolateral)</t>
         </is>
       </c>
       <c r="W8" t="n">
-        <v>40.5</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -2936,302 +2951,302 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>📖 PANDUAN METODOLOGI &amp; INTERPRETASI METRIK TERMAL (PPP, PPG, PGA)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="31" t="inlineStr">
         <is>
           <t>ThermalSight v1.8.3 • Diabetic Foot Thermal Biomechanics Evaluation Suite</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="32" t="inlineStr">
         <is>
           <t>1. TRIAD METRIK TERMAL TELAPAK KAKI (RINGKASAN EKSEKUTIF)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="33" t="inlineStr">
         <is>
           <t>Pilar</t>
         </is>
       </c>
-      <c r="B5" s="30" t="inlineStr">
+      <c r="B5" s="33" t="inlineStr">
         <is>
           <t>Metrik Singkat</t>
         </is>
       </c>
-      <c r="C5" s="30" t="inlineStr">
+      <c r="C5" s="33" t="inlineStr">
         <is>
           <t>Pertanyaan Inti</t>
         </is>
       </c>
-      <c r="D5" s="30" t="inlineStr">
+      <c r="D5" s="33" t="inlineStr">
         <is>
           <t>Karakteristik Data</t>
         </is>
       </c>
-      <c r="E5" s="30" t="inlineStr">
+      <c r="E5" s="33" t="inlineStr">
         <is>
           <t>Satuan</t>
         </is>
       </c>
-      <c r="F5" s="30" t="inlineStr">
+      <c r="F5" s="33" t="inlineStr">
         <is>
           <t>Formula Dasar</t>
         </is>
       </c>
-      <c r="G5" s="30" t="inlineStr">
+      <c r="G5" s="33" t="inlineStr">
         <is>
           <t>Fungsi Diagnostik</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>Pilar 1</t>
         </is>
       </c>
-      <c r="B6" s="31" t="inlineStr">
+      <c r="B6" s="34" t="inlineStr">
         <is>
           <t>PPP</t>
         </is>
       </c>
-      <c r="C6" s="32" t="inlineStr">
+      <c r="C6" s="35" t="inlineStr">
         <is>
           <t>Seberapa panas titik tersebut?</t>
         </is>
       </c>
-      <c r="D6" s="32" t="inlineStr">
+      <c r="D6" s="35" t="inlineStr">
         <is>
           <t>Nilai Suhu Absolut (Max, Min, Mean, Std)</t>
         </is>
       </c>
-      <c r="E6" s="31" t="inlineStr">
+      <c r="E6" s="34" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="F6" s="32" t="inlineStr">
+      <c r="F6" s="35" t="inlineStr">
         <is>
           <t>T_peak = max(T), T_mean = sum(T)/N</t>
         </is>
       </c>
-      <c r="G6" s="32" t="inlineStr">
+      <c r="G6" s="35" t="inlineStr">
         <is>
           <t>Mendeteksi hotspot fokal hiperemia &amp; skrining asimetri bilateral (ΔT &gt; 2.2°C).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="33" t="inlineStr">
+      <c r="A7" s="36" t="inlineStr">
         <is>
           <t>Pilar 2</t>
         </is>
       </c>
-      <c r="B7" s="33" t="inlineStr">
+      <c r="B7" s="36" t="inlineStr">
         <is>
           <t>PPG</t>
         </is>
       </c>
-      <c r="C7" s="34" t="inlineStr">
+      <c r="C7" s="37" t="inlineStr">
         <is>
           <t>Seberapa tajam beda suhunya?</t>
         </is>
       </c>
-      <c r="D7" s="34" t="inlineStr">
+      <c r="D7" s="37" t="inlineStr">
         <is>
           <t>Laju Kemiringan Spasial Gradien Suhu</t>
         </is>
       </c>
-      <c r="E7" s="33" t="inlineStr">
+      <c r="E7" s="36" t="inlineStr">
         <is>
           <t>°C/cm atau px</t>
         </is>
       </c>
-      <c r="F7" s="34" t="inlineStr">
+      <c r="F7" s="37" t="inlineStr">
         <is>
           <t>||∇T|| = sqrt(Gx^2 + Gy^2) [Sobel 2D]</t>
         </is>
       </c>
-      <c r="G7" s="34" t="inlineStr">
+      <c r="G7" s="37" t="inlineStr">
         <is>
           <t>Membedakan panas menyeluruh normal vs batas fokal peradangan akut/osteomielitis.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="31" t="inlineStr">
+      <c r="A8" s="34" t="inlineStr">
         <is>
           <t>Pilar 3</t>
         </is>
       </c>
-      <c r="B8" s="31" t="inlineStr">
+      <c r="B8" s="34" t="inlineStr">
         <is>
           <t>PGA</t>
         </is>
       </c>
-      <c r="C8" s="32" t="inlineStr">
+      <c r="C8" s="35" t="inlineStr">
         <is>
           <t>Ke mana arah menjalarnya panas?</t>
         </is>
       </c>
-      <c r="D8" s="32" t="inlineStr">
+      <c r="D8" s="35" t="inlineStr">
         <is>
           <t>Vektor Orientasi Disipasi Kalor</t>
         </is>
       </c>
-      <c r="E8" s="31" t="inlineStr">
+      <c r="E8" s="34" t="inlineStr">
         <is>
           <t>Derajat &amp; Kompas</t>
         </is>
       </c>
-      <c r="F8" s="32" t="inlineStr">
+      <c r="F8" s="35" t="inlineStr">
         <is>
           <t>θ = arctan2(Gy, Gx) % 360°</t>
         </is>
       </c>
-      <c r="G8" s="32" t="inlineStr">
+      <c r="G8" s="35" t="inlineStr">
         <is>
           <t>Memetakan arah rambatan perfusi vaskular ke arah distal jari atau proksimal tumit.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>2. ALASAN PEMILIHAN AREA ANATOMIS (T1, M1, M2) &amp; RADIUS 9×9</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="35" t="inlineStr">
+      <c r="A11" s="38" t="inlineStr">
         <is>
           <t>Titik Anatomis</t>
         </is>
       </c>
-      <c r="B11" s="35" t="inlineStr">
+      <c r="B11" s="38" t="inlineStr">
         <is>
           <t>Nama Wilayah</t>
         </is>
       </c>
-      <c r="C11" s="35" t="inlineStr">
+      <c r="C11" s="38" t="inlineStr">
         <is>
           <t>Zona Fisiologis</t>
         </is>
       </c>
-      <c r="D11" s="35" t="inlineStr">
+      <c r="D11" s="38" t="inlineStr">
         <is>
           <t>Alasan Pemilihan Klinis &amp; Biomekanika</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="36" t="inlineStr">
+      <c r="A12" s="39" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="B12" s="37" t="inlineStr">
+      <c r="B12" s="40" t="inlineStr">
         <is>
           <t>Hallux (Jempol Kaki)</t>
         </is>
       </c>
-      <c r="C12" s="36" t="inlineStr">
+      <c r="C12" s="39" t="inlineStr">
         <is>
           <t>Forefoot / Distal</t>
         </is>
       </c>
-      <c r="D12" s="38" t="inlineStr">
+      <c r="D12" s="41" t="inlineStr">
         <is>
           <t>Area kontak tumpuan akhir saat fase dorongan melangkah (push-off). Sangat rentan gesekan mekanis berulang dan mikrotrauma neuropatik.</t>
         </is>
       </c>
-      <c r="E12" s="39" t="n"/>
-      <c r="F12" s="39" t="n"/>
-      <c r="G12" s="39" t="n"/>
+      <c r="E12" s="42" t="n"/>
+      <c r="F12" s="42" t="n"/>
+      <c r="G12" s="42" t="n"/>
     </row>
     <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="36" t="inlineStr">
+      <c r="A13" s="39" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="B13" s="37" t="inlineStr">
+      <c r="B13" s="40" t="inlineStr">
         <is>
           <t>Caput Metatarsal 1</t>
         </is>
       </c>
-      <c r="C13" s="36" t="inlineStr">
+      <c r="C13" s="39" t="inlineStr">
         <is>
           <t>Forefoot / Medial</t>
         </is>
       </c>
-      <c r="D13" s="38" t="inlineStr">
+      <c r="D13" s="41" t="inlineStr">
         <is>
           <t>Titik tumpuan beban puncak tertinggi (peak plantar pressure) pada telapak kaki bagian dalam. Lokasi statistik nomor 1 kejadian ulkus diabetik.</t>
         </is>
       </c>
-      <c r="E13" s="39" t="n"/>
-      <c r="F13" s="39" t="n"/>
-      <c r="G13" s="39" t="n"/>
+      <c r="E13" s="42" t="n"/>
+      <c r="F13" s="42" t="n"/>
+      <c r="G13" s="42" t="n"/>
     </row>
     <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="36" t="inlineStr">
+      <c r="A14" s="39" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="B14" s="37" t="inlineStr">
+      <c r="B14" s="40" t="inlineStr">
         <is>
           <t>Caput Metatarsal 2</t>
         </is>
       </c>
-      <c r="C14" s="36" t="inlineStr">
+      <c r="C14" s="39" t="inlineStr">
         <is>
           <t>Forefoot / Central</t>
         </is>
       </c>
-      <c r="D14" s="38" t="inlineStr">
+      <c r="D14" s="41" t="inlineStr">
         <is>
           <t>Pusat distribusi arkus transversus. Area paling sering mengalami keruntuhan sendi metatarsal pada fase awal neuropatik Charcot Foot.</t>
         </is>
       </c>
-      <c r="E14" s="39" t="n"/>
-      <c r="F14" s="39" t="n"/>
-      <c r="G14" s="39" t="n"/>
+      <c r="E14" s="42" t="n"/>
+      <c r="F14" s="42" t="n"/>
+      <c r="G14" s="42" t="n"/>
     </row>
     <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="36" t="inlineStr">
+      <c r="A15" s="39" t="inlineStr">
         <is>
           <t>Radius 9×9</t>
         </is>
       </c>
-      <c r="B15" s="37" t="inlineStr">
+      <c r="B15" s="40" t="inlineStr">
         <is>
           <t>Standar Grid 81 Sel</t>
         </is>
       </c>
-      <c r="C15" s="36" t="inlineStr">
+      <c r="C15" s="39" t="inlineStr">
         <is>
           <t>1.2 cm Kontak Riil</t>
         </is>
       </c>
-      <c r="D15" s="38" t="inlineStr">
+      <c r="D15" s="41" t="inlineStr">
         <is>
           <t>Radius 4.5 sel (diameter 9 sel) dikunci dinamis ke skala fisik 1.2 cm. Menjamin flux termal setara antar pasien tanpa bias jarak kamera.</t>
         </is>
       </c>
-      <c r="E15" s="39" t="n"/>
-      <c r="F15" s="39" t="n"/>
-      <c r="G15" s="39" t="n"/>
+      <c r="E15" s="42" t="n"/>
+      <c r="F15" s="42" t="n"/>
+      <c r="G15" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
fix(workbench): refine Excel audit formulas, add regression test suite, and harden web/ipc pipeline
</commit_message>
<xml_diff>
--- a/example/bas_Result/PPP_PPG_PGA_Statistical_Summary.xlsx
+++ b/example/bas_Result/PPP_PPG_PGA_Statistical_Summary.xlsx
@@ -1906,7 +1906,7 @@
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>'=AVERAGE(D2:D22)</t>
+          <t>Formula: =AVERAGE(D2:D22)</t>
         </is>
       </c>
       <c r="E27" s="14">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>'=MAX(E2:E22)</t>
+          <t>Formula: =MAX(E2:E22)</t>
         </is>
       </c>
       <c r="E28" s="14">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>'=MIN(F2:F22)</t>
+          <t>Formula: =MIN(F2:F22)</t>
         </is>
       </c>
       <c r="E29" s="14">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>'=AVERAGE(H2:H22)</t>
+          <t>Formula: =AVERAGE(H2:H22)</t>
         </is>
       </c>
       <c r="E30" s="20">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>'=MAX(I2:I22)</t>
+          <t>Formula: =MAX(I2:I22)</t>
         </is>
       </c>
       <c r="E31" s="20">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="D34" s="25" t="inlineStr">
         <is>
-          <t>'=AVERAGE(M2:M22)</t>
+          <t>Formula: =AVERAGE(M2:M22)</t>
         </is>
       </c>
       <c r="E34" s="26">
@@ -2960,7 +2960,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>ThermalSight v1.8.3 • Diabetic Foot Thermal Biomechanics Evaluation Suite</t>
+          <t>ThermalSight v1.8.4 • Diabetic Foot Thermal Biomechanics Evaluation Suite</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3110,7 @@
       </c>
       <c r="F8" s="35" t="inlineStr">
         <is>
-          <t>θ = arctan2(Gy, Gx) % 360°</t>
+          <t>θ = arctan2(-Gy, Gx) % 360°</t>
         </is>
       </c>
       <c r="G8" s="35" t="inlineStr">

</xml_diff>